<commit_message>
Sample Testing targetting high NPV config
</commit_message>
<xml_diff>
--- a/backend_sample_testing/work_fair/output/submission_preview.xlsx
+++ b/backend_sample_testing/work_fair/output/submission_preview.xlsx
@@ -34,13 +34,13 @@
     <t>original_file_name</t>
   </si>
   <si>
-    <t>C:\Users\nikhi\Downloads\Doc-Forgery-Detector\test_backend\work_fair\input\2cd1b800-8443-4309-af6c-a733f7b92735.jpeg</t>
-  </si>
-  <si>
-    <t>2cd1b800-8443-4309-af6c-a733f7b92735.jpeg</t>
-  </si>
-  <si>
-    <t>C2||C3||C4||C7||C9</t>
+    <t>c:\Users\nikhi\Downloads\Doc-Forgery-Detector\backend_sample_testing\work_fair\input\1.png</t>
+  </si>
+  <si>
+    <t>1.png</t>
+  </si>
+  <si>
+    <t>C2||C3</t>
   </si>
 </sst>
 </file>
@@ -432,7 +432,7 @@
         <v>8</v>
       </c>
       <c r="D2">
-        <v>492</v>
+        <v>10</v>
       </c>
       <c r="E2">
         <v>1</v>

</xml_diff>